<commit_message>
Normalize workbook theme and property metadata at build time
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/artifacts/reconciliation.xlsx
+++ b/artifacts/reconciliation.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re226a2df4b8240ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="2" r:id="R904827f74f1c4a87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident Oracle" sheetId="3" r:id="R13dde7638d924677"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policy Results" sheetId="4" r:id="R7e5ac0e313af4680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R645f51512d3b4d56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="2" r:id="Rfd97cf9487254f58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incident Oracle" sheetId="3" r:id="Rc645a317cf744509"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policy Results" sheetId="4" r:id="Ra8a13885e2e846d1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -150,9 +150,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -202,7 +202,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>

</xml_diff>